<commit_message>
Create markers and annotations nodes
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Single-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Single-Agent.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -355,7 +355,7 @@
     <t xml:space="preserve">CAM02</t>
   </si>
   <si>
-    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT03/MULTICAMERA09</t>
+    <t xml:space="preserve">rtsp://127.0.0.1:8554/AGENT01/MULTICAMERA03</t>
   </si>
   <si>
     <t xml:space="preserve">Resolution [pix]</t>

</xml_diff>

<commit_message>
Fix multi-camera annotation issue
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Single-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Single-Agent.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -64,6 +64,9 @@
     <t xml:space="preserve">StartHour</t>
   </si>
   <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
     <t xml:space="preserve">MISSION00</t>
   </si>
   <si>
@@ -92,9 +95,6 @@
   </si>
   <si>
     <t xml:space="preserve">(16:30:00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
   </si>
   <si>
     <t xml:space="preserve">MISSION01</t>
@@ -607,17 +607,18 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="2" tint="-0.75"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">
@@ -711,7 +712,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -744,7 +745,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -756,12 +757,16 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -788,10 +793,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -801,10 +802,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1353,36 +1350,38 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8"/>
+      <c r="A3" s="8" t="s">
+        <v>11</v>
+      </c>
       <c r="B3" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
@@ -1431,9 +1430,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>21</v>
-      </c>
+      <c r="A4" s="13"/>
       <c r="B4" s="9" t="s">
         <v>22</v>
       </c>
@@ -1441,28 +1438,28 @@
         <v>23</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>24</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L4" s="12"/>
       <c r="M4" s="12"/>
@@ -1691,12 +1688,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -1718,7 +1715,7 @@
     </row>
     <row r="3" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>27</v>
@@ -1726,7 +1723,7 @@
       <c r="C3" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="15" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1740,7 +1737,7 @@
       <c r="C4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="15" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1780,15 +1777,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -1884,7 +1881,7 @@
       <c r="D3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="16" t="n">
         <v>2</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -1965,7 +1962,7 @@
       <c r="D4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>4</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2041,12 +2038,12 @@
         <v>48</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="16" t="n">
         <v>8</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -2127,7 +2124,7 @@
       <c r="D6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="16" t="n">
         <v>16</v>
       </c>
       <c r="F6" s="9" t="s">
@@ -2240,48 +2237,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>61</v>
       </c>
       <c r="L2" s="12"/>
@@ -2296,66 +2293,66 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="18" t="s">
+      <c r="C3" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="H3" s="18" t="n">
+      <c r="H3" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="19" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2407,32 +2404,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>74</v>
       </c>
       <c r="H2" s="12"/>
@@ -2448,22 +2445,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="18" t="n">
+      <c r="D3" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -2473,22 +2470,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -2560,56 +2557,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="17" t="s">
+      <c r="J2" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="18" t="s">
         <v>85</v>
       </c>
       <c r="M2" s="12"/>
@@ -2622,155 +2619,155 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="n">
+      <c r="J3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="18" t="n">
+      <c r="K3" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="19" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="H4" s="18" t="s">
+      <c r="H4" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="18" t="n">
+      <c r="J4" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="18" t="n">
+      <c r="K4" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="18" t="s">
+      <c r="L4" s="19" t="s">
         <v>100</v>
       </c>
       <c r="XFD4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="J5" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="K5" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="18" t="s">
+      <c r="L5" s="19" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="J6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="18" t="s">
+      <c r="L6" s="19" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2824,36 +2821,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="18" t="s">
         <v>112</v>
       </c>
       <c r="XEU2" s="3"/>
@@ -2868,48 +2865,48 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="19" t="s">
         <v>78</v>
       </c>
       <c r="D3" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="18" t="n">
+      <c r="G3" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>78</v>
       </c>
       <c r="D4" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="19" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="18" t="n">
+      <c r="G4" s="19" t="n">
         <v>0.583</v>
       </c>
     </row>
@@ -3294,7 +3291,7 @@
       <c r="C5" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="22" t="s">
         <v>155</v>
       </c>
       <c r="E5" s="22" t="s">

</xml_diff>

<commit_message>
Solve multi-camera annotation issue II
</commit_message>
<xml_diff>
--- a/src/flychams_common/config/Configuration-Single-Agent.xlsx
+++ b/src/flychams_common/config/Configuration-Single-Agent.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Mission" sheetId="1" state="visible" r:id="rId3"/>
@@ -544,7 +544,7 @@
     <numFmt numFmtId="165" formatCode="h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -605,13 +605,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -712,7 +705,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -745,7 +738,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -757,16 +750,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1430,7 +1419,7 @@
       <c r="BD3" s="12"/>
     </row>
     <row r="4" s="3" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
         <v>22</v>
       </c>
@@ -1549,92 +1538,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>163</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>145</v>
       </c>
       <c r="L2" s="12"/>
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="C3" s="22" t="b">
+      <c r="C3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="E3" s="22" t="b">
+      <c r="E3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1688,12 +1677,12 @@
   </cols>
   <sheetData>
     <row r="1" s="7" customFormat="true" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
       <c r="E1" s="12"/>
       <c r="XFB1" s="3"/>
       <c r="XFC1" s="3"/>
@@ -1723,7 +1712,7 @@
       <c r="C3" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="14" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1737,7 +1726,7 @@
       <c r="C4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1777,15 +1766,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -1881,7 +1870,7 @@
       <c r="D3" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="15" t="n">
         <v>2</v>
       </c>
       <c r="F3" s="9" t="s">
@@ -1962,7 +1951,7 @@
       <c r="D4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="15" t="n">
         <v>4</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -2043,7 +2032,7 @@
       <c r="D5" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="15" t="n">
         <v>8</v>
       </c>
       <c r="F5" s="9" t="s">
@@ -2124,7 +2113,7 @@
       <c r="D6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="15" t="n">
         <v>16</v>
       </c>
       <c r="F6" s="9" t="s">
@@ -2237,48 +2226,48 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>61</v>
       </c>
       <c r="L2" s="12"/>
@@ -2293,66 +2282,66 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="H3" s="19" t="n">
+      <c r="H3" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="H4" s="19" t="n">
+      <c r="H4" s="18" t="n">
         <v>300</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="19" t="n">
+      <c r="J4" s="18" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2404,32 +2393,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>74</v>
       </c>
       <c r="H2" s="12"/>
@@ -2445,22 +2434,22 @@
       <c r="XFD2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="19" t="n">
+      <c r="D3" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G3" s="2"/>
@@ -2470,22 +2459,22 @@
       <c r="XEY3" s="3"/>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="19" t="n">
+      <c r="D4" s="18" t="n">
         <v>0.2</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>0.8</v>
       </c>
       <c r="G4" s="2"/>
@@ -2557,56 +2546,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="17" t="s">
         <v>85</v>
       </c>
       <c r="M2" s="12"/>
@@ -2619,155 +2608,155 @@
       <c r="XFC2" s="12"/>
     </row>
     <row r="3" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="I3" s="19" t="n">
+      <c r="I3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="19" t="n">
+      <c r="J3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K3" s="19" t="n">
+      <c r="K3" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="18" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="4" s="12" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="I4" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J4" s="19" t="n">
+      <c r="I4" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K4" s="19" t="n">
+      <c r="K4" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L4" s="19" t="s">
+      <c r="L4" s="18" t="s">
         <v>100</v>
       </c>
       <c r="XFD4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="G5" s="19" t="s">
+      <c r="G5" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="I5" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="J5" s="19" t="n">
+      <c r="I5" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K5" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="L5" s="18" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="G6" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="J6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="19" t="n">
+      <c r="K6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="L6" s="18" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2821,36 +2810,36 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>112</v>
       </c>
       <c r="XEU2" s="3"/>
@@ -2865,48 +2854,48 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="19" t="n">
+      <c r="G3" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="18" t="n">
         <v>0.167</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
+      <c r="G4" s="18" t="n">
         <v>0.583</v>
       </c>
     </row>
@@ -2964,140 +2953,140 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="L2" s="21" t="s">
+      <c r="L2" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="M2" s="21" t="s">
+      <c r="M2" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="N2" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="O2" s="21" t="s">
+      <c r="O2" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="P2" s="20" t="s">
         <v>130</v>
       </c>
-      <c r="Q2" s="21" t="s">
+      <c r="Q2" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="R2" s="20" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="D3" s="22" t="n">
+      <c r="D3" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="22" t="n">
+      <c r="E3" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="F3" s="22" t="b">
+      <c r="F3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="H3" s="22" t="b">
+      <c r="H3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="I3" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="J3" s="22" t="b">
+      <c r="J3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="L3" s="22" t="b">
+      <c r="L3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="M3" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="N3" s="22" t="n">
+      <c r="N3" s="21" t="n">
         <v>6.5</v>
       </c>
-      <c r="O3" s="22" t="n">
+      <c r="O3" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="P3" s="22" t="n">
+      <c r="P3" s="21" t="n">
         <v>400</v>
       </c>
-      <c r="Q3" s="22" t="n">
+      <c r="Q3" s="21" t="n">
         <v>350</v>
       </c>
-      <c r="R3" s="22" t="n">
+      <c r="R3" s="21" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3157,52 +3146,52 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" s="7" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="J2" s="21" t="s">
+      <c r="J2" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="20" t="s">
         <v>145</v>
       </c>
       <c r="XFB2" s="3"/>
@@ -3210,110 +3199,110 @@
       <c r="XFD2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="G3" s="22" t="b">
+      <c r="G3" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="22" t="n">
+      <c r="K3" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="G4" s="22" t="b">
+      <c r="G4" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="G5" s="22" t="b">
+      <c r="G5" s="21" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="21" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>